<commit_message>
add fix for B06
</commit_message>
<xml_diff>
--- a/docs/project-tasks.xlsx
+++ b/docs/project-tasks.xlsx
@@ -267,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -363,6 +363,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -2681,7 +2684,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="69.75" customHeight="1" s="32">
+    <row r="7" ht="190" customHeight="1" s="32">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>B06</t>
@@ -2714,12 +2717,12 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Decide explicitly and record it: if the backend is the trust boundary, state that in an ADR and change no code; if it is not, carry the caller's identity (per-doctor keys, or a signed claim) and filter from that server-side rather than from the request.</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="inlineStr">
-        <is>
-          <t>Needs Decision</t>
+          <t>DECIDED AND CLOSED: the backend is the trust boundary. This service authenticates its caller and trusts it to decide which doctor may ask for what — already the recorded decision in ADR-0007, so no new ADR was written; a second copy of a decision only invites drift. No authorization was added. What did change is that the code no longer reads like access control when it is not: doctorId on GET /ingestions is documented as a filter with no user identity behind it to check against, and GET /patients/{patientId}/documents gains an optional doctorId filter of its own — needed now that the doctor is part of the document key (B05), because a patient seen by two doctors otherwise returns both doctors' transcripts with no way to narrow. Left optional rather than required: the patient's whole record is a legitimate thing for a trusted backend to ask for, and forcing a scope would narrow the endpoint's meaning. Covered by a test asserting unfiltered returns both doctors, filtered returns one, and an unknown doctor returns none.</t>
+        </is>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixes  B12 & B13
</commit_message>
<xml_diff>
--- a/docs/project-tasks.xlsx
+++ b/docs/project-tasks.xlsx
@@ -293,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -409,6 +409,9 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -2680,7 +2683,7 @@
           <t>FIXED. The defect was structural, not two missing calls: queueing and announcing were separate steps, so every path had to remember both. There is now one way in — IngestionQueue.EnqueueAsync announces and enqueues together — and all four call sites use it: fresh submit, retry endpoint, retry-via-resubmit, and startup recovery. IngestionsController no longer holds the channel or the publisher at all. Reruns carry only an ingestion id, so the doctor and patient come from a new GetIdentityAsync reading the record's own columns rather than deserializing the payload and its whole transcript. Startup recovery announces too: after a crash is exactly when someone is watching a bar that will not move. This also closed a latent ordering race — the old code published Queued AFTER writing to the channel, so a worker could announce Chunking before it; EnqueueAsync publishes first. Verified by disabling the publish: exactly the three announcement-dependent tests failed and the two that do not care kept passing.</t>
         </is>
       </c>
-      <c r="H5" s="34" t="inlineStr">
+      <c r="H5" s="40" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2722,7 +2725,7 @@
           <t>FIXED by decision: the document key is doctorId + patientId + sessionId + sequenceNumber, and all four are carried in the identifier itself (doctorId#patientId#sessionId#sequenceNumber). The id now answers 'whose document is this?' on its own, so DELETE /documents/{documentId} is safe without knowing whether session ids are globally unique — T25 is unblocked and no longer depends on the answer. Every query that asks whether two submissions are the same document matches on all four: in-flight detection, duplicate detection, the rerun staleness check, supersede, and the patient-list collapse (leave the doctor out of that last one and two doctors' transcripts of a session merge into one row). Stored chunk ids were rewritten by the DocumentIdCarriesDoctorAndPatient migration — a prefix prepend, no parsing. NOTE: putting the doctor in the key means two doctors filing the same patient, session and sequence hold two separate documents and neither supersedes the other — pinned by a test. Right if a session belongs to the doctor who recorded it; wrong if the same encounter can arrive under a different doctor account (locum, colleague re-filing a correction, or an unstable service account), where a correction would become a duplicate. Worth confirming with the backend team.</t>
         </is>
       </c>
-      <c r="H6" s="34" t="inlineStr">
+      <c r="H6" s="40" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2764,7 +2767,7 @@
           <t>DECIDED AND CLOSED: the backend is the trust boundary. This service authenticates its caller and trusts it to decide which doctor may ask for what — already the recorded decision in ADR-0007, so no new ADR was written; a second copy of a decision only invites drift. No authorization was added. What did change is that the code no longer reads like access control when it is not: doctorId on GET /ingestions is documented as a filter with no user identity behind it to check against, and GET /patients/{patientId}/documents gains an optional doctorId filter of its own — needed now that the doctor is part of the document key (B05), because a patient seen by two doctors otherwise returns both doctors' transcripts with no way to narrow. Left optional rather than required: the patient's whole record is a legitimate thing for a trusted backend to ask for, and forcing a scope would narrow the endpoint's meaning. Covered by a test asserting unfiltered returns both doctors, filtered returns one, and an unknown doctor returns none.</t>
         </is>
       </c>
-      <c r="H7" s="34" t="inlineStr">
+      <c r="H7" s="40" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2980,7 +2983,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="82.5" customHeight="1" s="32">
+    <row r="13" ht="171.75" customHeight="1" s="32">
       <c r="A13" s="35" t="inlineStr">
         <is>
           <t>B12</t>
@@ -3013,16 +3016,16 @@
       </c>
       <c r="G13" s="36" t="inlineStr">
         <is>
-          <t>Hash both sides before comparing (SHA-256 of the presented key against a precomputed digest of each valid key) so the compared values are always 32 bytes and the length of the secret cannot be observed at all. Then the comment is simply true.</t>
-        </is>
-      </c>
-      <c r="H13" s="38" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="95.25" customHeight="1" s="32">
+          <t>FIXED. The comparison now runs on SHA-256 digests rather than the keys themselves: two digests are always 32 bytes, so FixedTimeEquals never short-circuits on length and there is nothing left for the timing to expose. Every configured key is still checked even after one matches, for the same reason. Configuration is still read per request, which is what lets a rotated key take effect without a restart. The constant-time property is structural and not something a timing assertion could test without being flaky, so what the tests pin is the behaviour it must not have broken: six candidates — empty, one character, one short, one long, a valid key used as a prefix, and right length but wrong content — are all refused, and both rotation keys still work.</t>
+        </is>
+      </c>
+      <c r="H13" s="41" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="159" customHeight="1" s="32">
       <c r="A14" s="35" t="inlineStr">
         <is>
           <t>B13</t>
@@ -3055,12 +3058,12 @@
       </c>
       <c r="G14" s="36" t="inlineStr">
         <is>
-          <t>Refuse the combination at startup rather than discovering it under load: read MaxPoolSize and fail fast if WorkerCount leaves no headroom, the way the service already refuses to start without an API secret. Setting MaxPoolSize explicitly in the connection string would make the budget visible instead of implied.</t>
-        </is>
-      </c>
-      <c r="H14" s="38" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>FIXED. Program.cs now refuses to start when Ingestion:WorkerCount could claim more than half the connection pool, budgeting two connections per worker: the one carrying its advisory lock for the whole run, and one for the database work inside it. The message names both settings and says which to change. Checked at startup rather than discovered under load, because raising the worker count is the obvious thing to try when ingestion looks slow and the failure it caused would have been the service hanging with nothing in the logs to explain it — the same fail-fast treatment the missing API secret already gets. Verified by disabling the guard and confirming the test then reports no exception thrown.</t>
+        </is>
+      </c>
+      <c r="H14" s="41" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add fix for B08
</commit_message>
<xml_diff>
--- a/docs/project-tasks.xlsx
+++ b/docs/project-tasks.xlsx
@@ -202,34 +202,45 @@
     </font>
     <font>
       <name val="Arial"/>
+      <charset val="161"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF006100"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <charset val="161"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <charset val="161"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <charset val="161"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF9C6500"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <charset val="161"/>
+      <family val="2"/>
+      <b val="1"/>
       <color rgb="FF595959"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FF595959"/>
+      <color rgb="FF006100"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -293,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -385,35 +396,29 @@
     <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -784,13 +789,13 @@
   <dimension ref="B2:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" style="32" min="1" max="1"/>
-    <col width="46" customWidth="1" style="32" min="2" max="2"/>
-    <col width="12" customWidth="1" style="32" min="3" max="5"/>
-    <col width="14" customWidth="1" style="32" min="6" max="8"/>
+    <col width="3" customWidth="1" style="37" min="1" max="1"/>
+    <col width="46" customWidth="1" style="37" min="2" max="2"/>
+    <col width="12" customWidth="1" style="37" min="3" max="5"/>
+    <col width="14" customWidth="1" style="37" min="6" max="8"/>
   </cols>
   <sheetData>
-    <row r="2" ht="40.5" customHeight="1" s="32">
+    <row r="2" ht="40.5" customHeight="1" s="37">
       <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Clinical Document Ingestion Service - Developer Task List</t>
@@ -798,7 +803,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="31" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>Turns clinical documents (session transcripts first; doctor notes, lab PDFs, imaging reports next) into a patient-scoped, searchable knowledge store (Postgres + pgvector) for a future RAG chat. Only the existing backend calls this service. Stack: .NET 10, ASP.NET controllers, EF Core, Microsoft Agent Framework, SignalR. Work rule: take the first task whose dependencies are all Completed; each task is one red-green TDD cycle at the integration seam.</t>
         </is>
@@ -807,35 +812,35 @@
     <row r="4"/>
     <row r="5"/>
     <row r="6"/>
-    <row r="8" ht="31.5" customHeight="1" s="32">
+    <row r="8" ht="31.5" customHeight="1" s="37">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>The two invariants every task must preserve</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="38.25" customHeight="1" s="32">
-      <c r="B9" s="31" t="inlineStr">
+    <row r="9" ht="38.25" customHeight="1" s="37">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>1. The AI points, code copies - no generative model ever produces a stored number or word of patient text (ADR-0002/0006).</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="38.25" customHeight="1" s="32">
-      <c r="B10" s="31" t="inlineStr">
+    <row r="10" ht="38.25" customHeight="1" s="37">
+      <c r="B10" s="36" t="inlineStr">
         <is>
           <t>2. Nothing is ever partially visible - every ingestion commits atomically; corrections supersede in the same transaction (ADR-0003).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="25.5" customHeight="1" s="32">
-      <c r="B11" s="31" t="inlineStr">
+    <row r="11" ht="25.5" customHeight="1" s="37">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Full reasoning: docs/adr, docs/ingestion-pipeline-design.md, docs/prd.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" s="32">
+    <row r="13" ht="15.75" customHeight="1" s="37">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Status legend</t>
@@ -863,7 +868,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1" s="32">
+    <row r="18" ht="15.75" customHeight="1" s="37">
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Phases</t>
@@ -1080,16 +1085,16 @@
   <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" style="32" min="1" max="1"/>
-    <col width="24" customWidth="1" style="32" min="2" max="2"/>
-    <col width="30" customWidth="1" style="32" min="3" max="3"/>
-    <col width="66" customWidth="1" style="32" min="4" max="4"/>
-    <col width="54" customWidth="1" style="32" min="5" max="5"/>
-    <col width="11" customWidth="1" style="32" min="6" max="6"/>
-    <col width="13" customWidth="1" style="32" min="7" max="7"/>
+    <col width="7" customWidth="1" style="37" min="1" max="1"/>
+    <col width="24" customWidth="1" style="37" min="2" max="2"/>
+    <col width="30" customWidth="1" style="37" min="3" max="3"/>
+    <col width="66" customWidth="1" style="37" min="4" max="4"/>
+    <col width="54" customWidth="1" style="37" min="5" max="5"/>
+    <col width="11" customWidth="1" style="37" min="6" max="6"/>
+    <col width="13" customWidth="1" style="37" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.1" customHeight="1" s="32">
+    <row r="1" ht="26.1" customHeight="1" s="37">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>ID</t>
@@ -1126,7 +1131,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="38.25" customHeight="1" s="32">
+    <row r="2" ht="38.25" customHeight="1" s="37">
       <c r="A2" s="13" t="inlineStr">
         <is>
           <t>T01</t>
@@ -1159,7 +1164,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="38.25" customHeight="1" s="32">
+    <row r="3" ht="38.25" customHeight="1" s="37">
       <c r="A3" s="13" t="inlineStr">
         <is>
           <t>T02</t>
@@ -1196,7 +1201,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="51" customHeight="1" s="32">
+    <row r="4" ht="51" customHeight="1" s="37">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>T03</t>
@@ -1233,7 +1238,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38.25" customHeight="1" s="32">
+    <row r="5" ht="38.25" customHeight="1" s="37">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>T04</t>
@@ -1270,7 +1275,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="38.25" customHeight="1" s="32">
+    <row r="6" ht="38.25" customHeight="1" s="37">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>T05</t>
@@ -1307,7 +1312,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="51" customHeight="1" s="32">
+    <row r="7" ht="51" customHeight="1" s="37">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>T06</t>
@@ -1344,7 +1349,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="25.5" customHeight="1" s="32">
+    <row r="8" ht="25.5" customHeight="1" s="37">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>T07</t>
@@ -1381,7 +1386,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="25.5" customHeight="1" s="32">
+    <row r="9" ht="25.5" customHeight="1" s="37">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>T08</t>
@@ -1418,7 +1423,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="25.5" customHeight="1" s="32">
+    <row r="10" ht="25.5" customHeight="1" s="37">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>T09</t>
@@ -1455,7 +1460,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="63.75" customHeight="1" s="32">
+    <row r="11" ht="63.75" customHeight="1" s="37">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>T10</t>
@@ -1492,7 +1497,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="51" customHeight="1" s="32">
+    <row r="12" ht="51" customHeight="1" s="37">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>T11</t>
@@ -1529,7 +1534,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="38.25" customHeight="1" s="32">
+    <row r="13" ht="38.25" customHeight="1" s="37">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>T12</t>
@@ -1566,7 +1571,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="38.25" customHeight="1" s="32">
+    <row r="14" ht="38.25" customHeight="1" s="37">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>T13</t>
@@ -1603,7 +1608,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="51" customHeight="1" s="32">
+    <row r="15" ht="51" customHeight="1" s="37">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>T14</t>
@@ -1640,7 +1645,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="38.25" customHeight="1" s="32">
+    <row r="16" ht="38.25" customHeight="1" s="37">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>T15</t>
@@ -1677,7 +1682,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="38.25" customHeight="1" s="32">
+    <row r="17" ht="38.25" customHeight="1" s="37">
       <c r="A17" s="13" t="inlineStr">
         <is>
           <t>T16</t>
@@ -1714,7 +1719,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="38.25" customHeight="1" s="32">
+    <row r="18" ht="38.25" customHeight="1" s="37">
       <c r="A18" s="13" t="inlineStr">
         <is>
           <t>T17</t>
@@ -1751,7 +1756,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="38.25" customHeight="1" s="32">
+    <row r="19" ht="38.25" customHeight="1" s="37">
       <c r="A19" s="13" t="inlineStr">
         <is>
           <t>T18</t>
@@ -1788,7 +1793,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="38.25" customHeight="1" s="32">
+    <row r="20" ht="38.25" customHeight="1" s="37">
       <c r="A20" s="13" t="inlineStr">
         <is>
           <t>T19</t>
@@ -1825,7 +1830,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="38.25" customHeight="1" s="32">
+    <row r="21" ht="38.25" customHeight="1" s="37">
       <c r="A21" s="13" t="inlineStr">
         <is>
           <t>T20</t>
@@ -1862,7 +1867,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="38.25" customHeight="1" s="32">
+    <row r="22" ht="38.25" customHeight="1" s="37">
       <c r="A22" s="13" t="inlineStr">
         <is>
           <t>T21</t>
@@ -1899,7 +1904,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="38.25" customHeight="1" s="32">
+    <row r="23" ht="38.25" customHeight="1" s="37">
       <c r="A23" s="13" t="inlineStr">
         <is>
           <t>T22</t>
@@ -1936,7 +1941,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="25.5" customHeight="1" s="32">
+    <row r="24" ht="25.5" customHeight="1" s="37">
       <c r="A24" s="13" t="inlineStr">
         <is>
           <t>T23</t>
@@ -1973,7 +1978,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="25.5" customHeight="1" s="32">
+    <row r="25" ht="25.5" customHeight="1" s="37">
       <c r="A25" s="13" t="inlineStr">
         <is>
           <t>T24</t>
@@ -2010,7 +2015,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="38.25" customHeight="1" s="32">
+    <row r="26" ht="38.25" customHeight="1" s="37">
       <c r="A26" s="13" t="inlineStr">
         <is>
           <t>T25</t>
@@ -2047,7 +2052,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="38.25" customHeight="1" s="32">
+    <row r="27" ht="38.25" customHeight="1" s="37">
       <c r="A27" s="13" t="inlineStr">
         <is>
           <t>T26</t>
@@ -2084,7 +2089,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="51" customHeight="1" s="32">
+    <row r="28" ht="51" customHeight="1" s="37">
       <c r="A28" s="13" t="inlineStr">
         <is>
           <t>T27</t>
@@ -2121,7 +2126,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="38.25" customHeight="1" s="32">
+    <row r="29" ht="38.25" customHeight="1" s="37">
       <c r="A29" s="13" t="inlineStr">
         <is>
           <t>T28</t>
@@ -2158,7 +2163,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="51" customHeight="1" s="32">
+    <row r="30" ht="51" customHeight="1" s="37">
       <c r="A30" s="13" t="inlineStr">
         <is>
           <t>T29</t>
@@ -2195,7 +2200,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="38.25" customHeight="1" s="32">
+    <row r="31" ht="38.25" customHeight="1" s="37">
       <c r="A31" s="13" t="inlineStr">
         <is>
           <t>T30</t>
@@ -2232,7 +2237,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="63.75" customHeight="1" s="32">
+    <row r="32" ht="63.75" customHeight="1" s="37">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>T31</t>
@@ -2269,7 +2274,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="25.5" customHeight="1" s="32">
+    <row r="33" ht="25.5" customHeight="1" s="37">
       <c r="A33" s="13" t="inlineStr">
         <is>
           <t>T32</t>
@@ -2306,7 +2311,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="63.75" customHeight="1" s="32">
+    <row r="34" ht="63.75" customHeight="1" s="37">
       <c r="A34" s="13" t="inlineStr">
         <is>
           <t>T33</t>
@@ -2343,7 +2348,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="25.5" customHeight="1" s="32">
+    <row r="35" ht="25.5" customHeight="1" s="37">
       <c r="A35" s="13" t="inlineStr">
         <is>
           <t>T34</t>
@@ -2380,7 +2385,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="63.75" customHeight="1" s="32">
+    <row r="36" ht="63.75" customHeight="1" s="37">
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>T35</t>
@@ -2417,7 +2422,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="38.25" customHeight="1" s="32">
+    <row r="37" ht="38.25" customHeight="1" s="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
           <t>T36</t>
@@ -2469,17 +2474,17 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" style="32" min="1" max="1"/>
-    <col width="22" customWidth="1" style="32" min="2" max="2"/>
-    <col width="34" customWidth="1" style="32" min="3" max="3"/>
-    <col width="11" customWidth="1" style="32" min="4" max="4"/>
-    <col width="64" customWidth="1" style="32" min="5" max="5"/>
-    <col width="48" customWidth="1" style="32" min="6" max="6"/>
-    <col width="64" customWidth="1" style="32" min="7" max="7"/>
-    <col width="15" customWidth="1" style="32" min="8" max="8"/>
+    <col width="7" customWidth="1" style="37" min="1" max="1"/>
+    <col width="22" customWidth="1" style="37" min="2" max="2"/>
+    <col width="34" customWidth="1" style="37" min="3" max="3"/>
+    <col width="11" customWidth="1" style="37" min="4" max="4"/>
+    <col width="64" customWidth="1" style="37" min="5" max="5"/>
+    <col width="48" customWidth="1" style="37" min="6" max="6"/>
+    <col width="64" customWidth="1" style="37" min="7" max="7"/>
+    <col width="15" customWidth="1" style="37" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.1" customHeight="1" s="32">
+    <row r="1" ht="26.1" customHeight="1" s="37">
       <c r="A1" s="17" t="inlineStr">
         <is>
           <t>ID</t>
@@ -2521,7 +2526,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="120.75" customHeight="1" s="32">
+    <row r="2" ht="120.75" customHeight="1" s="37">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>B01</t>
@@ -2563,7 +2568,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="174.95" customHeight="1" s="32">
+    <row r="3" ht="174.95" customHeight="1" s="37">
       <c r="A3" s="18" t="inlineStr">
         <is>
           <t>B02</t>
@@ -2605,7 +2610,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="174.95" customHeight="1" s="32">
+    <row r="4" ht="174.95" customHeight="1" s="37">
       <c r="A4" s="18" t="inlineStr">
         <is>
           <t>B03</t>
@@ -2647,7 +2652,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="190" customHeight="1" s="32">
+    <row r="5" ht="189.95" customHeight="1" s="37">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>B04</t>
@@ -2683,13 +2688,13 @@
           <t>FIXED. The defect was structural, not two missing calls: queueing and announcing were separate steps, so every path had to remember both. There is now one way in — IngestionQueue.EnqueueAsync announces and enqueues together — and all four call sites use it: fresh submit, retry endpoint, retry-via-resubmit, and startup recovery. IngestionsController no longer holds the channel or the publisher at all. Reruns carry only an ingestion id, so the doctor and patient come from a new GetIdentityAsync reading the record's own columns rather than deserializing the payload and its whole transcript. Startup recovery announces too: after a crash is exactly when someone is watching a bar that will not move. This also closed a latent ordering race — the old code published Queued AFTER writing to the channel, so a worker could announce Chunking before it; EnqueueAsync publishes first. Verified by disabling the publish: exactly the three announcement-dependent tests failed and the two that do not care kept passing.</t>
         </is>
       </c>
-      <c r="H5" s="40" t="inlineStr">
+      <c r="H5" s="31" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="190" customHeight="1" s="32">
+    <row r="6" ht="189.95" customHeight="1" s="37">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>B05</t>
@@ -2725,13 +2730,13 @@
           <t>FIXED by decision: the document key is doctorId + patientId + sessionId + sequenceNumber, and all four are carried in the identifier itself (doctorId#patientId#sessionId#sequenceNumber). The id now answers 'whose document is this?' on its own, so DELETE /documents/{documentId} is safe without knowing whether session ids are globally unique — T25 is unblocked and no longer depends on the answer. Every query that asks whether two submissions are the same document matches on all four: in-flight detection, duplicate detection, the rerun staleness check, supersede, and the patient-list collapse (leave the doctor out of that last one and two doctors' transcripts of a session merge into one row). Stored chunk ids were rewritten by the DocumentIdCarriesDoctorAndPatient migration — a prefix prepend, no parsing. NOTE: putting the doctor in the key means two doctors filing the same patient, session and sequence hold two separate documents and neither supersedes the other — pinned by a test. Right if a session belongs to the doctor who recorded it; wrong if the same encounter can arrive under a different doctor account (locum, colleague re-filing a correction, or an unstable service account), where a correction would become a duplicate. Worth confirming with the backend team.</t>
         </is>
       </c>
-      <c r="H6" s="40" t="inlineStr">
+      <c r="H6" s="31" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="190" customHeight="1" s="32">
+    <row r="7" ht="189.95" customHeight="1" s="37">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>B06</t>
@@ -2767,13 +2772,13 @@
           <t>DECIDED AND CLOSED: the backend is the trust boundary. This service authenticates its caller and trusts it to decide which doctor may ask for what — already the recorded decision in ADR-0007, so no new ADR was written; a second copy of a decision only invites drift. No authorization was added. What did change is that the code no longer reads like access control when it is not: doctorId on GET /ingestions is documented as a filter with no user identity behind it to check against, and GET /patients/{patientId}/documents gains an optional doctorId filter of its own — needed now that the doctor is part of the document key (B05), because a patient seen by two doctors otherwise returns both doctors' transcripts with no way to narrow. Left optional rather than required: the patient's whole record is a legitimate thing for a trusted backend to ask for, and forcing a scope would narrow the endpoint's meaning. Covered by a test asserting unfiltered returns both doctors, filtered returns one, and an unknown doctor returns none.</t>
         </is>
       </c>
-      <c r="H7" s="40" t="inlineStr">
+      <c r="H7" s="31" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="57" customHeight="1" s="32">
+    <row r="8" ht="57" customHeight="1" s="37">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>B07</t>
@@ -2809,13 +2814,13 @@
           <t>Send to a group keyed by doctorId, with clients joining their own group on connect, so routing is enforced by the hub rather than by the consumer's good behaviour.</t>
         </is>
       </c>
-      <c r="H8" s="25" t="inlineStr">
-        <is>
-          <t>Needs Decision</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="82.5" customHeight="1" s="32">
+      <c r="H8" s="38" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="190" customHeight="1" s="37">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>B08</t>
@@ -2848,16 +2853,16 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Add documentId (and sessionId / sequenceNumber) to the event payload, and confirm the shape with the backend team before they build against the current one.</t>
-        </is>
-      </c>
-      <c r="H9" s="25" t="inlineStr">
-        <is>
-          <t>Needs Decision</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="69.75" customHeight="1" s="32">
+          <t>FIXED by decision: events now carry documentId and sessionId, and the resync list carries documentId too, so both halves of the gap are closed. PublishAsync was changed to take the whole IngestionIdentity rather than loose ids, which means a caller cannot announce a stage while leaving out what the stage is about — the shape of the call enforces it rather than the discipline of whoever adds the next one. IngestionIdentity gained the document's parts and assembles the id itself, so events, the resync list and the patient document list all name a document identically and no consumer rebuilds the string. Two incidental improvements: the failure path now reads the record's own columns instead of deserializing the stored payload — announcing a failure no longer opens a whole transcript to find two strings — and the resync query materializes before assembling ids, since that is C# no database can run. Verified by setting the id to a wrong value: exactly the three assertions that depend on it failed, and nothing else did.</t>
+        </is>
+      </c>
+      <c r="H9" s="39" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="69.75" customHeight="1" s="37">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>B09</t>
@@ -2899,7 +2904,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="95.25" customHeight="1" s="32">
+    <row r="11" ht="95.25" customHeight="1" s="37">
       <c r="A11" s="27" t="inlineStr">
         <is>
           <t>B10</t>
@@ -2941,127 +2946,127 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="190" customHeight="1" s="32">
-      <c r="A12" s="35" t="inlineStr">
+    <row r="12" ht="189.95" customHeight="1" s="37">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>B11</t>
         </is>
       </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>Chunking / Robustness</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>A truncated code fence crashes chunk-plan parsing</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
+      <c r="D12" s="34" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="E12" s="33" t="inlineStr">
         <is>
           <t>StripCodeFences assumes a fenced response is closed. When the model returns an opening fence with no closing one, LastIndexOf("```") finds the opening fence itself, so the slice runs from after the first newline back to index 0 and throws ArgumentOutOfRangeException. Reproduced directly: '```json\n{"chunks":[{"startLine":0' throws "length ('-8') must be a non-negative value".</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
+      <c r="F12" s="33" t="inlineStr">
         <is>
           <t>The throw is an ArgumentOutOfRangeException, which the surrounding catch (JsonException) does not catch — so it escapes RequestChunkPlanAsync and the ONE corrective retry designed for exactly this case never runs. The ingestion fails with a message about a negative length, which tells a doctor nothing and points an engineer at the wrong place. The likely trigger is an answer cut off at the output-token limit, which a long transcript makes more likely, not less.</t>
         </is>
       </c>
-      <c r="G12" s="36" t="inlineStr">
+      <c r="G12" s="33" t="inlineStr">
         <is>
           <t>FIXED. StripCodeFences now removes the opening fence first and looks for a closing one only in what remains, so it can never find the opening fence and slice backwards. A response with no closing fence is handed to the parser whole, fails as unreadable JSON, and reaches the corrective retry the design always intended for a bad answer. The method no longer throws for any input, null included, so the narrow catch (JsonException) was kept rather than widened — a bad answer from the model is expected and handled, a defect in our own code should still be loud. Bonus: a plan whose closing fence the model merely forgot is now read successfully instead of discarded, since nothing but the fence was missing. Three tests: a truncated answer gets its retry and completes; two truncated answers fail naming the model rather than a string index; an unclosed but complete plan is read with no retry at all. Edge cases re-checked separately — fence-only, empty, null, and a ``` sequence inside a JSON string value.</t>
         </is>
       </c>
-      <c r="H12" s="40" t="inlineStr">
+      <c r="H12" s="31" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="171.75" customHeight="1" s="32">
-      <c r="A13" s="35" t="inlineStr">
+    <row r="13" ht="171.75" customHeight="1" s="37">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>B12</t>
         </is>
       </c>
-      <c r="B13" s="36" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>API key comparison reveals the length of a valid key</t>
         </is>
       </c>
-      <c r="D13" s="39" t="inlineStr">
+      <c r="D13" s="35" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="E13" s="33" t="inlineStr">
         <is>
           <t>The handler compares with CryptographicOperations.FixedTimeEquals, whose fixed-time guarantee holds only for equal-length inputs — it returns false immediately when lengths differ. The comment beside it says the comparison is fixed time so that timing cannot narrow the secret, which is true of the content but not of the length.</t>
         </is>
       </c>
-      <c r="F13" s="36" t="inlineStr">
+      <c r="F13" s="33" t="inlineStr">
         <is>
           <t>An attacker who can time requests can learn how long a valid key is, narrowing a brute-force search. Small on its own, and the keys are long random secrets, but the code states a property it does not quite have — which is how a reviewer stops looking.</t>
         </is>
       </c>
-      <c r="G13" s="36" t="inlineStr">
+      <c r="G13" s="33" t="inlineStr">
         <is>
           <t>FIXED. The comparison now runs on SHA-256 digests rather than the keys themselves: two digests are always 32 bytes, so FixedTimeEquals never short-circuits on length and there is nothing left for the timing to expose. Every configured key is still checked even after one matches, for the same reason. Configuration is still read per request, which is what lets a rotated key take effect without a restart. The constant-time property is structural and not something a timing assertion could test without being flaky, so what the tests pin is the behaviour it must not have broken: six candidates — empty, one character, one short, one long, a valid key used as a prefix, and right length but wrong content — are all refused, and both rotation keys still work.</t>
         </is>
       </c>
-      <c r="H13" s="41" t="inlineStr">
+      <c r="H13" s="31" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="159" customHeight="1" s="32">
-      <c r="A14" s="35" t="inlineStr">
+    <row r="14" ht="159" customHeight="1" s="37">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>B13</t>
         </is>
       </c>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>Worker / Configuration</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>WorkerCount can exceed the connection pool and deadlock startup</t>
         </is>
       </c>
-      <c r="D14" s="39" t="inlineStr">
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E14" s="36" t="inlineStr">
+      <c r="E14" s="33" t="inlineStr">
         <is>
           <t>Introduced by the B03 fix: every in-flight ingestion now holds a dedicated Npgsql connection for the whole run, to keep its advisory lock alive, on top of the connections EF uses. Ingestion:WorkerCount is configurable and the connection string sets no MaxPoolSize, so the ceiling is Npgsql's default of 100 shared between both.</t>
         </is>
       </c>
-      <c r="F14" s="36" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Harmless at the default of 4. Raise WorkerCount toward 100 — the obvious lever when ingestion looks slow — and workers exhaust the pool holding locks while EF waits for a connection that only they can release. It would present as the service hanging under load, with nothing in the logs naming the cause.</t>
         </is>
       </c>
-      <c r="G14" s="36" t="inlineStr">
+      <c r="G14" s="33" t="inlineStr">
         <is>
           <t>FIXED. Program.cs now refuses to start when Ingestion:WorkerCount could claim more than half the connection pool, budgeting two connections per worker: the one carrying its advisory lock for the whole run, and one for the database work inside it. The message names both settings and says which to change. Checked at startup rather than discovered under load, because raising the worker count is the obvious thing to try when ingestion looks slow and the failure it caused would have been the service hanging with nothing in the logs to explain it — the same fail-fast treatment the missing API secret already gets. Verified by disabling the guard and confirming the test then reports no exception thrown.</t>
         </is>
       </c>
-      <c r="H14" s="41" t="inlineStr">
+      <c r="H14" s="31" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>

</xml_diff>

<commit_message>
add known bugs to the list
</commit_message>
<xml_diff>
--- a/docs/project-tasks.xlsx
+++ b/docs/project-tasks.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$G$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Known Bugs'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Known Bugs'!$A$1:$H$17</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -251,6 +251,20 @@
     <font>
       <b val="1"/>
       <color rgb="FF9C0006"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FF595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF9C6500"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -314,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -435,6 +449,15 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -2487,7 +2510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="37" min="1" max="1"/>
@@ -3130,8 +3153,92 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="184.5" customHeight="1" s="37">
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>B15</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>Chunking / Quality</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>Splitting an oversized chunk can leave a fragment below the size floor</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>ChunkSizeGuardrails.Apply is SplitOversized(MergeUndersized(...)), so the merge pass runs before the split and never sees what the split produces. LastLineOfNextPart recomputes an even-size target for each part, which reduces starved tails but does not prevent one: a short trailing line falls through as a part of its own. Demonstrated end to end at the test thresholds (floor 12 tokens, ceiling 40) with three lines of 156/156/8 characters submitted as a single planned chunk — the stored chunks came out at 39, 39 and 2 tokens. (ChunkSizeGuardrails.cs)</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>A 2-token chunk is precisely what the floor exists to prevent: it carries almost no retrievable meaning and occupies a retrieval slot a fuller chunk would have used. The damage is bounded — a split part inherits its parent range's context blurb, so what gets embedded is not literally three words — which makes this retrieval quality rather than correctness. The sharper problem is that the comment on LastLineOfNextPart states the guarantee outright ('so a split never leaves a starved tail that the merge pass would undo'), and a comment claiming a property the code does not have is how a reviewer stops looking. B12 read the same way.</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="inlineStr">
+        <is>
+          <t>Fold a final part that lands below the floor back into the part before it, inside the same original chunk. That is a local fix with an obvious termination argument, and it accepts a part slightly over the ceiling — already the documented trade, since verbatim completeness outranks both limits. Resist the tidier-looking 'run merge and split to a fixed point': merging is allowed to push a chunk over the ceiling, so a naive loop of the two passes has no termination argument. Whatever is done, weaken the comment to what the code actually promises. Worth taking alongside other chunking work rather than on its own.</t>
+        </is>
+      </c>
+      <c r="H16" s="43" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="184.5" customHeight="1" s="37">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>B16</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>Domain / Identity</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>documentId joins unvalidated ids with '#' and has no inverse</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>DocumentIdentity.For joins doctorId, patientId, sessionId and sequenceNumber with '#', and IngestionRequestValidation excludes that character from none of them. doctorId 'a' with patientId 'b#c' and doctorId 'a#b' with patientId 'c' therefore assemble the same identifier. DocumentIdentity has For and no inverse. (PatientDocument.cs)</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>Nothing is corrupt today: every query asking whether two submissions are the same document matches on the columns rather than on the assembled string, and the chunk delete still carries the patient-scoped predicate B05 deliberately kept. It becomes real with T25, DELETE /documents/{documentId}, which receives the identifier alone and must split it back into four parts — and would then either refuse legitimate ids or address the wrong document. That is the very endpoint B05's key decision was made to unblock, so the question B05 answered is only half settled: the id carries its whole scope, but not unambiguously.</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>Settle it before T25 is written rather than during. Cheapest is to reject '#' in doctorId, patientId and sessionId at IngestionRequestValidation: the existing format then parses with a plain split, at the cost of constraining identifiers the backend owns — so it needs the backend team's agreement, and belongs in the same conversation as the doctorId question B05 left open. Otherwise encode each part before joining (percent- or base64url-encoding), which needs nobody's agreement but rewrites every stored chunk id and so needs a migration like the one B05 already required. Either way add DocumentIdentity.Parse next to For, so the round trip lives in one place and the delete endpoint cannot invent its own.</t>
+        </is>
+      </c>
+      <c r="H17" s="43" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:H17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add agent instructions in the database
</commit_message>
<xml_diff>
--- a/docs/project-tasks.xlsx
+++ b/docs/project-tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\medical-assistance\medicalassistant\ai-med\medical-assistance-ai\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98326FA1-B36A-4221-B492-24F90281C34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51219FD8-039C-4ACA-9068-3AF5A7DBFE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1922,11 +1922,11 @@
       </c>
       <c r="D26" s="9">
         <f>COUNTIFS(Tasks!$B$2:$B$999,B26,Tasks!$G$2:$G$999,"Completed")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="9">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.25">
@@ -1956,11 +1956,11 @@
       </c>
       <c r="D28" s="11">
         <f>SUM(D20:D27)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E28" s="11">
         <f>SUM(E20:E27)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -2646,8 +2646,8 @@
       <c r="F29" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="G29" s="16" t="s">
-        <v>9</v>
+      <c r="G29" s="41" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
add document summary and patient rolling summary
</commit_message>
<xml_diff>
--- a/docs/project-tasks.xlsx
+++ b/docs/project-tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\medical-assistance\medicalassistant\ai-med\medical-assistance-ai\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B0F875-0A94-4790-BA96-BD046889EB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090B3B6C-2C5B-4228-B807-E47959ED8D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -1959,11 +1959,11 @@
       </c>
       <c r="D27" s="9">
         <f>COUNTIFS(Tasks!$B$2:$B$999,B27,Tasks!$G$2:$G$999,"Completed")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" s="9">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.25">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="D28" s="11">
         <f>SUM(D20:D27)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E28" s="11">
         <f>SUM(E20:E27)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2804,8 +2804,8 @@
       <c r="F35" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="G35" s="16" t="s">
-        <v>9</v>
+      <c r="G35" s="45" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>